<commit_message>
Harden LNNCP dashboard workbook to avoid Excel repair-on-open issues
Removed custom chart line dash-style/width overrides and Font objects
embedded inside conditional-formatting rules -- both are known
openpyxl edge cases that can trigger Excel's "we found a problem with
some content" repair dialog even though the underlying zip/XML is
technically valid. Conditional formatting now uses fill color only.
Verified: valid zip, every XML/rels part in the archive parses
cleanly, and openpyxl reloads all 5 sheets without error.
</commit_message>
<xml_diff>
--- a/hybrid/outputs/lnncp_early_warning_dashboard.xlsx
+++ b/hybrid/outputs/lnncp_early_warning_dashboard.xlsx
@@ -131,13 +131,8 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="5">
     <dxf>
-      <font>
-        <b val="1"/>
-        <color rgb="00006100"/>
-        <sz val="18"/>
-      </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00C6EFCE"/>
@@ -145,11 +140,6 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <b val="1"/>
-        <color rgb="009C6500"/>
-        <sz val="18"/>
-      </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00FFEB9C"/>
@@ -157,11 +147,6 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <b val="1"/>
-        <color rgb="009C5700"/>
-        <sz val="18"/>
-      </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00FFD599"/>
@@ -169,11 +154,6 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <b val="1"/>
-        <color rgb="009C0006"/>
-        <sz val="18"/>
-      </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00FFC7CE"/>
@@ -181,62 +161,6 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <b val="1"/>
-        <color rgb="00808080"/>
-        <sz val="18"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00E7E6E6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="00006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00C6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="009C6500"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00FFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="009C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00FFD599"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color rgb="009C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00FFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="00808080"/>
-      </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00E7E6E6"/>
@@ -347,7 +271,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="15000">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -380,7 +304,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="10000">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -414,7 +338,7 @@
           </tx>
           <spPr>
             <a:ln>
-              <a:prstDash val="dash"/>
+              <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
@@ -447,7 +371,7 @@
           </tx>
           <spPr>
             <a:ln>
-              <a:prstDash val="dash"/>
+              <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
@@ -50658,19 +50582,19 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="Q2:Q644">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="5">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"NORMAL"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="6">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
       <formula>"WATCH"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="7">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
       <formula>"EARLY WARNING"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="8">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
       <formula>"CRITICAL"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="9">
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
       <formula>"Insufficient History"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>